<commit_message>
File confidential WasteWerx IP-Protected brochure into the record (SRC-019)
Filed the IP-protected WasteWerx brochure into 07_PARTNERS_AND_ROLES/05_WasteWerx
and 01_SOURCE_FILES/05_Original_Technology_Files (named CONFIDENTIAL), with a
handling note (partner-facing only; do not publish proprietary specs/reactor
photos; WasteWerx owns IP, mutual NDA 5/18). Logged as SRC-019 in the VAULT
Workbook Source Register and rebuilt the workbook. Refreshed the corridor zip.

https://claude.ai/code/session_01NNVRfcBeiW4jRftzrwemzW
</commit_message>
<xml_diff>
--- a/docs/business/casespace/00_CONTROL/Michigan_LTC_VAULT_Workbook.xlsx
+++ b/docs/business/casespace/00_CONTROL/Michigan_LTC_VAULT_Workbook.xlsx
@@ -3344,7 +3344,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I22"/>
+  <dimension ref="A1:I23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4262,6 +4262,53 @@
       <c r="I22" s="4" t="inlineStr">
         <is>
           <t>10-yr, 40,000 t/yr at $25/ton tipping</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>SRC-019</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>WasteWerx Brochure (IP-Protected)</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>07_PARTNERS_AND_ROLES/05_WasteWerx</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>Technology brochure</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="F23" s="4" t="inlineStr">
+        <is>
+          <t>WasteWerx</t>
+        </is>
+      </c>
+      <c r="G23" s="4" t="inlineStr">
+        <is>
+          <t>ON FILE — CONFIDENTIAL</t>
+        </is>
+      </c>
+      <c r="H23" s="4" t="inlineStr">
+        <is>
+          <t>Technology / partner packet</t>
+        </is>
+      </c>
+      <c r="I23" s="4" t="inlineStr">
+        <is>
+          <t>IP-protected version; partner-facing only; do NOT publish proprietary specs/reactor photos (NDA 5/18)</t>
         </is>
       </c>
     </row>

</xml_diff>